<commit_message>
Regenerate sample data with exclusive BU-aligned prescriptions
Key changes to generate_sample_data.py:
- 100 HCPs (was 50): exactly 3 AIR + 5 SBU + 2 Vaccines per territory
  so every territory (including T002 for rlee) has HCPs in each BU
- BU-exclusive specialty assignment: AIR=Neurology+Oncology,
  SBU=Psychiatry+IM+Geriatrics, Vaccines=FP+Cardiology
- BU-aligned prescriptions: each HCP only writes scripts for their
  BU products (Neurologists/Oncologists -> NEXOLID+VERITONEX only;
  Psychiatrists/IM/Geriatrics -> CLAROZEPT+DEPTRAZOL only;
  Vaccines HCPs -> zero pharma prescriptions)
- Calls now routed to BU-appropriate product IDs per HCP specialty
- Speakers certified for their BU products only
- KPI_Territory gains CLAROZEPT_NRx + DEPTRAZOL_NRx columns

Result: 0 HCP overlap across BUs; distinct TRx/NRx per BU per territory;
no rep sees another BUs data.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sourcedata/Dim_Products.xlsx
+++ b/sourcedata/Dim_Products.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CNS/Psychiatry</t>
+          <t>CNS/Neurology</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CNS/Psychiatry</t>
+          <t>CNS/Neurology</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CNS/Psychiatry</t>
+          <t>CNS/Neurology</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CNS/Psychiatry</t>
+          <t>CNS/Neurology</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">

</xml_diff>